<commit_message>
update xlsx 2026-07-09 05:55
</commit_message>
<xml_diff>
--- a/dm_data_2026-06.xlsx
+++ b/dm_data_2026-06.xlsx
@@ -50,9 +50,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,40 +520,40 @@
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>0.9607867702330243</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>0.9946624803767661</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>0.9959183673469387</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>1.682817155402227</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="4" t="n">
         <v>24771</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="4" t="n">
         <v>18416</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="4" t="n">
         <v>8350</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="2" t="n">
         <v>0.7434500020184893</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="2" t="n">
         <v>0.4534100781928758</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="2" t="n">
         <v>0.3370877235476969</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="5" t="n">
         <v>877.7305065868262</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="2" t="n">
         <v>0.02747895678192049</v>
       </c>
     </row>
@@ -564,40 +568,40 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>0.9649191959006701</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>0.9877358490566037</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>0.994811320754717</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>17.28756868131868</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="4" t="n">
         <v>2536</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="4" t="n">
         <v>1491</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="4" t="n">
         <v>627</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="2" t="n">
         <v>0.5879337539432177</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="2" t="n">
         <v>0.420523138832998</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="2" t="n">
         <v>0.2472397476340694</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="5" t="n">
         <v>1145.495901116427</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="2" t="n">
         <v>0.03978702222666533</v>
       </c>
     </row>
@@ -612,40 +616,40 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>0.9646424721523535</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>0.9980151156576837</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>0.9981677990686312</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>0.1641834759576202</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="4" t="n">
         <v>14507</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="4" t="n">
         <v>10847</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="4" t="n">
         <v>4929</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="2" t="n">
         <v>0.7477080030330185</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="2" t="n">
         <v>0.4544113579791648</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="2" t="n">
         <v>0.3397670090301234</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="5" t="n">
         <v>813.9730594441064</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="2" t="n">
         <v>0.02385594407535814</v>
       </c>
     </row>
@@ -660,40 +664,40 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>0.9529553679131484</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>0.9967436352871522</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>0.9972370238800079</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>0.1385955370974653</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="4" t="n">
         <v>7693</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="4" t="n">
         <v>6046</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="4" t="n">
         <v>2776</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="2" t="n">
         <v>0.785909268165865</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="2" t="n">
         <v>0.4591465431690374</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="2" t="n">
         <v>0.3608475237228649</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="5" t="n">
         <v>933.3815814121034</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="2" t="n">
         <v>0.02868833736936087</v>
       </c>
     </row>
@@ -708,40 +712,40 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>0.7878787878787878</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>0.5984251968503937</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>0.6771653543307087</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="3" t="n">
         <v>13.1609756097561</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="2" t="n">
         <v>0.9142857142857143</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="2" t="n">
         <v>0.5625</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="2" t="n">
         <v>0.5142857142857142</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="5" t="n">
         <v>426.8511111111113</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="2" t="n">
         <v>0.02602266180142116</v>
       </c>
     </row>
@@ -859,46 +863,46 @@
           <t>总计</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>0.9594473245992577</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>0.9957793704723732</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>0.9967397855414215</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>1.457738495253085</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="4" t="n">
         <v>23122</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="4" t="n">
         <v>17009</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="4" t="n">
         <v>7971</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="2" t="n">
         <v>0.735619756076464</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="2" t="n">
         <v>0.4686342524545828</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="2" t="n">
         <v>0.3447366144797163</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="5" t="n">
         <v>766.9640544067175</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="2" t="n">
         <v>0.02543034129906833</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="4" t="n">
         <v>34257228</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2" s="4" t="n">
         <v>871173</v>
       </c>
     </row>
@@ -908,46 +912,46 @@
           <t>EF成人英语课程咨询 - 小F</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>0.9646424721523535</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>0.9980151156576837</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>0.9981677990686312</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>0.1641834759576202</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="4" t="n">
         <v>14507</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="4" t="n">
         <v>10847</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="4" t="n">
         <v>4929</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="2" t="n">
         <v>0.7477080030330185</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="2" t="n">
         <v>0.4544113579791648</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="2" t="n">
         <v>0.3397670090301234</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="5" t="n">
         <v>813.973059444106</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="2" t="n">
         <v>0.02385594407535814</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="4" t="n">
         <v>21900328</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3" s="4" t="n">
         <v>522453</v>
       </c>
     </row>
@@ -957,46 +961,46 @@
           <t>EF成人英语课程咨询 - 小E</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>0.9475661548513558</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>0.9963695543314972</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>0.9969954932398598</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>0.1622841132438423</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="4" t="n">
         <v>6284</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="4" t="n">
         <v>4862</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="4" t="n">
         <v>2397</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="2" t="n">
         <v>0.7737110120942076</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="2" t="n">
         <v>0.493006993006993</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="2" t="n">
         <v>0.3814449395289625</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="5" t="n">
         <v>676.8194817171241</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="2" t="n">
         <v>0.02623695722839398</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="4" t="n">
         <v>10075025</v>
       </c>
-      <c r="O4" t="n">
+      <c r="O4" s="4" t="n">
         <v>264338</v>
       </c>
     </row>
@@ -1006,46 +1010,46 @@
           <t>EF成人英语培训</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>0.9617557583659279</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>0.9860950173812283</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>0.9918887601390498</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>17.19526760563381</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="4" t="n">
         <v>2296</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="4" t="n">
         <v>1268</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="4" t="n">
         <v>627</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="2" t="n">
         <v>0.5522648083623694</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="2" t="n">
         <v>0.4944794952681388</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="2" t="n">
         <v>0.2730836236933798</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="5" t="n">
         <v>751.798484848485</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="2" t="n">
         <v>0.03708016684305988</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="4" t="n">
         <v>2261047</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" s="4" t="n">
         <v>83840</v>
       </c>
     </row>
@@ -1055,46 +1059,46 @@
           <t>EF成人英语广东中心</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="2" t="n">
         <v>0.7878787878787878</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>0.5984251968503937</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>0.6771653543307087</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>13.1609756097561</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="2" t="n">
         <v>0.9142857142857143</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="2" t="n">
         <v>0.5625</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="2" t="n">
         <v>0.5142857142857142</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="5" t="n">
         <v>426.8511111111112</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="2" t="n">
         <v>0.02602266180142116</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="4" t="n">
         <v>20828</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="4" t="n">
         <v>542</v>
       </c>
     </row>

</xml_diff>